<commit_message>
Edit phase 1 materials as a student report
</commit_message>
<xml_diff>
--- a/Фаза 1 - Выбор концепции проекта/Данные и расчёты/Фаза 1 Экспертные оценки.xlsx
+++ b/Фаза 1 - Выбор концепции проекта/Данные и расчёты/Фаза 1 Экспертные оценки.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Итог" sheetId="1" r:id="Reebc177b496d44d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOPSIS" sheetId="2" r:id="R5772c2d5d0ca448e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="МАИ" sheetId="3" r:id="Re9ffbf52c8874cbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Эксперт 1" sheetId="4" r:id="R507dc540d3af41ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Эксперт 2" sheetId="5" r:id="Ra9e61ce8e5c9478f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Эксперт 3" sheetId="6" r:id="R3f4fc016b4d24825"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Эксперт 4" sheetId="7" r:id="R13416bf388d54029"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Итог" sheetId="1" r:id="R2090a2ecc86e4a61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOPSIS" sheetId="2" r:id="R2adddde3245b44bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="МАИ" sheetId="3" r:id="Re4031962696c458c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Эксперт 1" sheetId="4" r:id="R029828f6c2644e83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Эксперт 2" sheetId="5" r:id="Re144f0266c2c447a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Эксперт 3" sheetId="6" r:id="Rd93ac47167314f92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Эксперт 4" sheetId="7" r:id="Rd4816d513bf044b5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -357,7 +357,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="2" t="str">
-        <x:v>Фаза 1 — модельные экспертные оценки</x:v>
+        <x:v>Фаза 1 — исходные оценки и результаты</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -367,12 +367,12 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="str">
-        <x:v>Как заполнить</x:v>
+        <x:v>Состав расчёта</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="38" customHeight="1">
       <x:c r="A5" s="4" t="str">
-        <x:v>1. Четыре листа заполнены модельными профилями M1–M4. Это не личные ответы студентов.</x:v>
+        <x:v>Исходные значения заданы четырьмя сценарными профилями M1–M4; опрос участников не проводился.</x:v>
       </x:c>
       <x:c r="B5" s="4"/>
       <x:c r="C5" s="4"/>
@@ -382,7 +382,7 @@
     </x:row>
     <x:row r="6" ht="38" customHeight="1">
       <x:c r="A6" s="4" t="str">
-        <x:v>2. Для TOPSIS приведены три числа по шкале 1–9: осторожная, ожидаемая и благоприятная оценки.</x:v>
+        <x:v>TOPSIS: трёхточечные оценки по шкале 1–9 — осторожная, ожидаемая, благоприятная.</x:v>
       </x:c>
       <x:c r="B6" s="4"/>
       <x:c r="C6" s="4"/>
@@ -392,7 +392,7 @@
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
       <x:c r="A7" s="4" t="str">
-        <x:v>3. Для МАИ приведены независимые парные сравнения; число показывает предпочтение первого элемента.</x:v>
+        <x:v>МАИ: парные сравнения критериев и альтернатив на шкале Саати.</x:v>
       </x:c>
       <x:c r="B7" s="4"/>
       <x:c r="C7" s="4"/>
@@ -402,7 +402,7 @@
     </x:row>
     <x:row r="8" ht="38" customHeight="1">
       <x:c r="A8" s="4" t="str">
-        <x:v>4. Листы TOPSIS и МАИ показывают промежуточные таблицы и формулы, связанные с четырьмя анкетами.</x:v>
+        <x:v>Расчётные листы TOPSIS и МАИ связаны формулами с четырьмя листами исходных оценок.</x:v>
       </x:c>
       <x:c r="B8" s="4"/>
       <x:c r="C8" s="4"/>
@@ -412,7 +412,7 @@
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
       <x:c r="A9" s="4" t="str">
-        <x:v>5. Изменение оценок в анкете пересчитывает результаты в этой книге при открытии в Excel.</x:v>
+        <x:v>Лист «Итог» отражает результаты обоих методов для заданных исходных значений.</x:v>
       </x:c>
       <x:c r="B9" s="4"/>
       <x:c r="C9" s="4"/>
@@ -422,7 +422,7 @@
     </x:row>
     <x:row r="10" ht="38" customHeight="1">
       <x:c r="A10" s="4" t="str">
-        <x:v>6. По заданию требуется команда из трёх человек; состав из четырёх следует согласовать с преподавателем.</x:v>
+        <x:v>Фактический состав команды — четыре человека; в тексте задания указаны три.</x:v>
       </x:c>
       <x:c r="B10" s="4"/>
       <x:c r="C10" s="4"/>
@@ -552,7 +552,7 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="6" t="str">
-        <x:v>Результаты модельного расчёта</x:v>
+        <x:v>Результаты сравнения</x:v>
       </x:c>
       <x:c r="B27" s="6"/>
       <x:c r="C27" s="6"/>
@@ -3554,7 +3554,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="10" t="str">
-        <x:v>Индивидуальная анкета эксперта</x:v>
+        <x:v>Оценки сценарного профиля M1</x:v>
       </x:c>
       <x:c r="B1" s="10"/>
       <x:c r="C1" s="10"/>
@@ -3565,7 +3565,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>Модельный профиль</x:v>
+        <x:v>Сценарный профиль</x:v>
       </x:c>
       <x:c r="B3" t="str">
         <x:v>M1 — Акцент на практической пользе и понятном пользовательском сценарии</x:v>
@@ -3573,7 +3573,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>Смоделировано для демонстрации метода; не является ответом участника команды.</x:v>
+        <x:v>Сценарные исходные значения; индивидуальный опрос участников не проводился.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -4103,7 +4103,7 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" t="str">
-        <x:v>В D укажите предпочтение первого элемента перед вторым: от 1/9 до 9.</x:v>
+        <x:v>Столбец D: предпочтение первого элемента относительно второго, от 1/9 до 9.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -4690,7 +4690,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="10" t="str">
-        <x:v>Индивидуальная анкета эксперта</x:v>
+        <x:v>Оценки сценарного профиля M2</x:v>
       </x:c>
       <x:c r="B1" s="10"/>
       <x:c r="C1" s="10"/>
@@ -4701,7 +4701,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>Модельный профиль</x:v>
+        <x:v>Сценарный профиль</x:v>
       </x:c>
       <x:c r="B3" t="str">
         <x:v>M2 — Акцент на полезности и простоте запуска</x:v>
@@ -4709,7 +4709,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>Смоделировано для демонстрации метода; не является ответом участника команды.</x:v>
+        <x:v>Сценарные исходные значения; индивидуальный опрос участников не проводился.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -5239,7 +5239,7 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" t="str">
-        <x:v>В D укажите предпочтение первого элемента перед вторым: от 1/9 до 9.</x:v>
+        <x:v>Столбец D: предпочтение первого элемента относительно второго, от 1/9 до 9.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -5826,7 +5826,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="10" t="str">
-        <x:v>Индивидуальная анкета эксперта</x:v>
+        <x:v>Оценки сценарного профиля M3</x:v>
       </x:c>
       <x:c r="B1" s="10"/>
       <x:c r="C1" s="10"/>
@@ -5837,7 +5837,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>Модельный профиль</x:v>
+        <x:v>Сценарный профиль</x:v>
       </x:c>
       <x:c r="B3" t="str">
         <x:v>M3 — Акцент на реализуемости учебной командой</x:v>
@@ -5845,7 +5845,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>Смоделировано для демонстрации метода; не является ответом участника команды.</x:v>
+        <x:v>Сценарные исходные значения; индивидуальный опрос участников не проводился.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -6375,7 +6375,7 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" t="str">
-        <x:v>В D укажите предпочтение первого элемента перед вторым: от 1/9 до 9.</x:v>
+        <x:v>Столбец D: предпочтение первого элемента относительно второго, от 1/9 до 9.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -6962,7 +6962,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="10" t="str">
-        <x:v>Индивидуальная анкета эксперта</x:v>
+        <x:v>Оценки сценарного профиля M4</x:v>
       </x:c>
       <x:c r="B1" s="10"/>
       <x:c r="C1" s="10"/>
@@ -6973,7 +6973,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>Модельный профиль</x:v>
+        <x:v>Сценарный профиль</x:v>
       </x:c>
       <x:c r="B3" t="str">
         <x:v>M4 — Акцент на пригодности для последующих фаз планирования</x:v>
@@ -6981,7 +6981,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>Смоделировано для демонстрации метода; не является ответом участника команды.</x:v>
+        <x:v>Сценарные исходные значения; индивидуальный опрос участников не проводился.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -7511,7 +7511,7 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" t="str">
-        <x:v>В D укажите предпочтение первого элемента перед вторым: от 1/9 до 9.</x:v>
+        <x:v>Столбец D: предпочтение первого элемента относительно второго, от 1/9 до 9.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">

</xml_diff>